<commit_message>
Refactor templates and add new modals for manual processing and contract/discount reviews
- Updated concept_review.html to change warning message text.
- Modified index.html to include a manual processing modal and adjust flash message handling.
- Enhanced result.html to include processing issues modal and updated warning message text.
- Created desktop_app.py to initialize and run the application with a GUI.
- Added money.py for monetary value handling and allocation functions.
- Introduced runtime.py for application runtime management and resource handling.
- Added _manual_processing_modal.html and _processing_issues_modal.html for user notifications.
- Created contract_review.html and discount_review.html for handling contract and discount validations.
</commit_message>
<xml_diff>
--- a/Diccionario_Conceptos_Simple.xlsx
+++ b/Diccionario_Conceptos_Simple.xlsx
@@ -497,7 +497,11 @@
           <t>SEGUN_CONTRATO</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CUOTA ADMON GENERAL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -601,7 +605,11 @@
           <t>1537210003</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>FONDO DE IMPREVISTOS</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: Add warnings panel template and associated tests for process warnings
</commit_message>
<xml_diff>
--- a/Diccionario_Conceptos_Simple.xlsx
+++ b/Diccionario_Conceptos_Simple.xlsx
@@ -514,7 +514,11 @@
           <t>1537210004</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CuotadeAdministración, CANON DE ARRENDAMIENTO GRAVADO, CUOTA DE ADMINISTRACION PUBLICIDAD (P Y P), MODULO AIRE ACONDICIONADO ( C ), MODULO PUBLICIDAD (A), PUBLICIDADO</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -527,7 +531,11 @@
           <t>1532001600</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>AREAS COMUNES L2, ARRENDAMIENTO ESPACIO VENTAS AL DETALLE FIJO OCO, CANON DE ARRENDAMIENTO GRAVADO CANON DE ARRENDAMIENTO DEL DE DE EL TESORO LOCAL 1738- 202607, CUOTA DE PUBLICIDAD, ENERGIA Contador 10101325 Lectura Ant.43, 758 Lectura Act.43, 798 Consumo 40 Factor 1, EXPENSAS, FONDO DE PROMOCION LOCALES, INTERESES DE MORA GRAVADOS FACTURA No. S93665, INTERESES POR MORA, MODULO GENERAL, PUBLICIDAD, RECOLECCION DE ASEO CC, SERVICIO DE ACUEDUCTO DE LOCALES</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -540,7 +548,11 @@
           <t>1532001605</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>AIRE ACONDICIONADO, ARRENDAMIENTOS IVA 19%, CONCESION DE ESPACIO FIJO LOCALES, CUOTA DE ADMINISTRACION PPTO GASTOS (PG), ENERGIA Contador 10101330 Lectura Ant.96, 584 Lectura Act.98, 061 Consumo 1, 477 Factor 1, EXPENSAS COMUNES, FONDO DE RESERVA, SERV PARA USO Y APROVEC DEL INMUEB LOCALES</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -553,7 +565,11 @@
           <t>1532001604</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION RECIBIDA PARA TERCEROS, CONSUMO ENERGIA TORRES, MANTO A.A. PLANTA EMERG</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -566,7 +582,11 @@
           <t>1532001800</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CONTRIBUCION AREA COMUN L2 GRAVADA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -579,7 +599,11 @@
           <t>1532001600</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ARRENDAMIENTO LOCAL 252 CC ANDINO, ENERGIA Contador 10101359 Lectura Ant.79, 735 Lectura Act.81, 521 Consumo 1, 786 Factor 1, INTERESES ADMINISTRACIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -592,7 +616,11 @@
           <t>1245150017</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ACUEDUCTO Y ALCANTARILLADO Contador 9346402 Lectura Ant.3, 500.358 Lectura Act.3, 500.524 Consumo .166 Factor 1, ADMINISTRACIÓN CENTRO COMERCIAL (E), CIUDADELA COMERCIAL UNICENTRO LOCAL 2185, CUOTA DE ADMINISTRACION</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -607,7 +635,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>FONDO DE IMPREVISTOS</t>
+          <t>FONDO DE IMPREVISTOS, Canon de Arrendamiento, RECUPERACION DE COSTOS Y DEDUCCIONES ACUEDUCTO ZONA L2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor learning dictionary phrase handling and enhance validation
- Updated `_append_learning_dictionary_phrases` to support encoded account selection and improved error handling for invalid concepts and phrases.
- Modified HTML templates to streamline form submission with processing indicators and improved search functionality in warnings panel.
- Added unit tests for concept dictionary saving and expense tax code logic, ensuring robust validation and handling of various scenarios.
- Enhanced prorateo matching tests to cover edge cases and ensure accurate vendor and store rate application.
</commit_message>
<xml_diff>
--- a/Diccionario_Conceptos_Simple.xlsx
+++ b/Diccionario_Conceptos_Simple.xlsx
@@ -3,15 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diccionario'!$A$1:$C$11</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,32 +24,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,42 +41,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9E2F3"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9E2F3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9E2F3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9E2F3"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,254 +413,447 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="130" customWidth="1" min="3" max="3"/>
+    <col width="56.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.33203125" customWidth="1" min="2" max="2"/>
+    <col width="84.33203125" customWidth="1" min="3" max="3"/>
+    <col width="23.77734375" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>GL Account</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Frases/palabras</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Sigla</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>RENTA</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>SEGUN_CONTRATO</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CUOTA ADMON GENERAL</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CONSTRUCCIONES Y EDIFICACIONES RICA 11, 04, 1 ARRENDAMIENTOS, ARIENDO LOC.1328 CCIAL. PREMIUM PLAZA, 01 AL 31, ARRENDAMIENTOS IVA 19%, CIUDADELA COMERCIAL UNICENTRO LOCAL 2185, CanonArrendamientoVariabl, ARRENDAMIENTO BIEN INMUEBLE LOCAL COMERCIAL, ARRENDAMIENTO VARIABLE, Arrendamiento LOCAL 511 Y 544 CHIPICHAPE CALI, Arriendo inmueble local 2-014 A Centro comercial Titan, CANON DE ARRENDAMIENTO 25 LOCAL 1180 UBICADO EN LA AV CRA 15 12430 CENTRO COMERCIAL UNICENTRO EN BOGOTA DEL 10 DE AL 09, CANON DE ARRENDAMIENTO 25% LOCAL 1-180, UBICADO EN LA CRA. 15 124-30 DEL CENTRO COMERCIAL UNICENTRO, EN BOGOTÁ, CANON DE ARRENDAMIENTO GRAVADO local 118-119 CC Unicentro Girardot, CANON DE ARRENDAMIENTO GRAVADO locales 133 y 134 CC Unicentro Villavicencio, CANON, Canon de Arrendamiento, Canon de arrendamiento correspondiente desde el uno (1) de al treinta y uno (31) de según nuevo canon de arrendamiento pactado de los locales comerciales No, y depósitos No. 43 y 44 ubicados en el centro comercial y depósitos negocios andino. Propietario Prevesa SAS. F Louis C SAS con NIT 901821682-4, actúa como mandatario en la facturación de ingresos, por cuenta de terceros del mandante Prevesa SAS con NIT No. 900.062.970-2 quién será beneficiario de pago y de los efectos tributarios de dicha factura, ARRENDAMIENTO ESPACIO VENTAS AL DETALLE FIJO OCO, ARRENDAMIENTO LOCAL 252 CC ANDINO BOGOTA, ARRENDAMIENTO LOCAL COMERCIAL, SERV PARA USO Y APROVEC DEL INMUEB LOCALES, ARRIENDO LOCAL # 1246 DEL COMPLEJO COMERCIAL CHIA, UBICADO EN LA AV PRADILLA 900 ESTE DEL MUNICIPIO DE CHIA, 30 dias Arrendamiento de Inm 1372026 KR 15 No. 93 60 LC 117, ARRENDAMIENTO, ARRENDAMIENTO INMUEBLE-CC IMPERIAL LC 107, ARRENDAMIENTO INMUEBLES - LOCAL (+IR), ARRENDAMIENTO LOCAL 1150 CC SANTA FE MEDELLIN 7 A 7, ARRENDAMIENTO LOCAL 2 106, ARRIENDO 1 AL 30, ARRIENDO LC N1-60 C.CIAL P. PRADO, ARRIENDO LOCAL 1180 UNICENTRO, Arrendamiento Local 260 Salitre Plaza, situado en la Cra. 68B # 14-39 correspondiente al de /2.026, Descuento Comercial Arriendo, RETROACTIVO, VALOR MINIMO MENSUAL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RENTA</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>INTERES</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>1537210004</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>CuotadeAdministración, CANON DE ARRENDAMIENTO GRAVADO, CUOTA DE ADMINISTRACION PUBLICIDAD (P Y P), MODULO AIRE ACONDICIONADO ( C ), MODULO PUBLICIDAD (A), PUBLICIDADO</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>INTERESES DE MORA GMO PPA-36029 PPA-36281, INTERESES CUOTA DE ADMON, INTERESES DE MORA, INTERESES ADMINISTRACIÓN, Cobro de pena incumplimiento - sanción moratoria - Tarifa: 5 %, INT DE MORA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>INTERES</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>VIGILANCIA</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>1532001600</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>AREAS COMUNES L2, ARRENDAMIENTO ESPACIO VENTAS AL DETALLE FIJO OCO, CANON DE ARRENDAMIENTO GRAVADO CANON DE ARRENDAMIENTO DEL DE DE EL TESORO LOCAL 1738- 202607, CUOTA DE PUBLICIDAD, ENERGIA Contador 10101325 Lectura Ant.43, 758 Lectura Act.43, 798 Consumo 40 Factor 1, EXPENSAS, FONDO DE PROMOCION LOCALES, INTERESES DE MORA GRAVADOS FACTURA No. S93665, INTERESES POR MORA, MODULO GENERAL, PUBLICIDAD, RECOLECCION DE ASEO CC, SERVICIO DE ACUEDUCTO DE LOCALES</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VIGILANCIA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ENERGIA</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>1532001605</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>AIRE ACONDICIONADO, ARRENDAMIENTOS IVA 19%, CONCESION DE ESPACIO FIJO LOCALES, CUOTA DE ADMINISTRACION PPTO GASTOS (PG), ENERGIA Contador 10101330 Lectura Ant.96, 584 Lectura Act.98, 061 Consumo 1, 477 Factor 1, EXPENSAS COMUNES, FONDO DE RESERVA, SERV PARA USO Y APROVEC DEL INMUEB LOCALES</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ReembolsogastoSSPPEnergí, MANDATO EPM ENERGIA, CONSUMO ENERGIA TORRES, RECOBRO DE ENERGIA B-201 CORRESPONDIENTE DEL AL ; LI: 87557.96 Kwh, LF: 90249.37 Kwh, CONSUMO 2691.41 Kwh, RECOBRO DE ENERGIA L-109 CORRESPONDIENTE DEL AL ; LI: 169451.48 Kwh, LF: 171309.06 Kwh, CONSUMO 1857.58 Kwh, VALOR MODULO ENERGIA TORRES Y MTO. A.A, EXP.COMUNES DE PLANTAS ELECTRICAS, ENERGIA Contador 10101325 Lectura Ant.43, 798 Lectura Act.45, 069.5 Consumo 1, 271.5 Factor 1, ENERGIA Contador 10101328 Lectura Ant.74, 013 Lectura Act.74, 013.3 Consumo .3 Factor 1, ENERGIA Contador 10101330 Lectura Ant.98, 061 Lectura Act.99, 506.5 Consumo 1, 445.5 Factor 1, ENERGIA Contador 10101359 Lectura Ant.81, 521 Lectura Act.83, 199.8 Consumo 1, 678.8 Factor 1, RECOBRO DE ENERGIA B-201 CORRESPONDIENTE DEL AL ; LI: 90249.37 Kwh, LF: 92964.6 Kwh, CONSUMO 2715.23 Kwh, RECOBRO DE ENERGIA L-109 CORRESPONDIENTE DEL AL ; LI: 171309.06 Kwh, LF: 173284.23 Kwh, CONSUMO 1975.17 Kwh, ReembolsogastoSSPPEnergí, ENERGIA Contador 10101330 Lectura Ant.96, 584 Lectura Act.98, 061 Consumo 1, 477 Factor 1, ENERGIA Contador 10101359 Lectura Ant.79, 735 Lectura Act.81, 521 Consumo 1, 786 Factor 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ENERGIA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>ACUED</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>1532001604</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>ADMINISTRACION RECIBIDA PARA TERCEROS, CONSUMO ENERGIA TORRES, MANTO A.A. PLANTA EMERG</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>REINTEGRO SERVICIO DE ACUEDUCTO, ACUEDUCTO, ReembolsogastoSSPPAcuedu, REINTEGRO CONSUMO DE AGUAContador 496718 Lectura Ant.96.78 Lectura Act.97.24 Consumo .46 Factor 1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ACUED</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>MTTO</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>1532001800</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>CONTRIBUCION AREA COMUN L2 GRAVADA</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MANTO A.A. PLANTA EMERG</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MTTO</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>ASEO/AIRE</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AIRE</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>1532001600</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>ARRENDAMIENTO LOCAL 252 CC ANDINO, ENERGIA Contador 10101359 Lectura Ant.79, 735 Lectura Act.81, 521 Consumo 1, 786 Factor 1, INTERESES ADMINISTRACIÓN</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MODULO D: AIRE ACONDICIONADO ETAPA II, AIRE ACONDICIONADO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>AIRE</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ASEO</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>1532001600</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>REINTEGRO SERVICIO DE ASEO, VIGILANCIA, REINTEGRO DE ASEO, RECOLECCION DE ASEO CC, FUMIGACIÓN</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ASEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>1245150017</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>ACUEDUCTO Y ALCANTARILLADO Contador 9346402 Lectura Ant.3, 500.358 Lectura Act.3, 500.524 Consumo .166 Factor 1, ADMINISTRACIÓN CENTRO COMERCIAL (E), CIUDADELA COMERCIAL UNICENTRO LOCAL 2185, CUOTA DE ADMINISTRACION</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CUOTA DE ADMINISTRACION, GENERAL - ADMINISTRACION, 01 CUOTA DE ADMON-EXPENSAS, ADM GC %, ADMON, ADMON X C INQ. LC PROPIO, CUOTA COMUNES NECESARIAS I AGO26, CUOTA COMUNES NECESARIAS II AGO26, CUOTA DE FONDOS DE IMPREVISTO, EXPENSAS, EXPENSAS COMUNES, GASTO COMÚN, GASTO COMÚN /2026OC, Suma Minima, Garantizada, Suma Minima Garantizada, ADMINISTRACION, FONDO DE IMPREVISTO, MODULO GENERAL, CONCESION DE ESPACIO FIJO LOCALES, ADMINISTRACION RECIBIDA PARA TERCEROS, CONCESION MINIMO /2026OC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>1537210003</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>FONDO DE IMPREVISTOS, Canon de Arrendamiento, RECUPERACION DE COSTOS Y DEDUCCIONES ACUEDUCTO ZONA L2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>GV</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MODULO C: MERCADEO O PUBLICIDAD, FONDO DE PROMOCION LOCALES, 02 CUOTA DE ADMON-PUBLICIDAD, CUOTA DE PUBLICIDAD, PUBLICIDAD, PUBLICIDADO, EXP.COMUNES DE MERCADEO, MODULO COMERCIAL, Descuento Comercial Fondo Promo, FONDO DE PROMOCION SOBRE EL VALOR MINIMO MENSUAL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GC V</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>1537210002</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cuota de administración de propiedad horizontal, GC v, DESCUENTO POR PRONTO PAGO C CIAL, Cuota de Admón Concesión, VALOR MODULO COPROPIEDAD, AREAS COMUNES L2, CONTRIBUCION AREA COMUN L2 GRAVADA, EXCESO DE VENTAS (+IR), FONDO DE IMPREVISTOS, GMO L111 JARDIN PLAZA CALI, Administracion</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GC V</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PARQUEADERO</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>1532002507</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PARQUEADEROS</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PARQUEADERO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RECU PRIM POLIZA</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>1532002509</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:C11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="150" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Instrucciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Cada fila tiene Concepto, GL Account y todas las frases/palabras que identifican ese concepto, separadas por coma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>El usuario puede cambiar el GL Account directamente en este archivo si negocio confirma otra cuenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Cuando el usuario agregue una frase nueva, la app debe agregarla a la fila del concepto elegido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Para evitar confusiones, la app debe evaluar primero las frases mas largas/completas. Ejemplo: RETROACTIVO EXPENSAS debe ganar sobre EXPENSAS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>RENTA usa GL Account SEGUN_CONTRATO: VIGENTE/POR VENCER = RF 1245150017; CESADO/CERRADA = RV 1537210004; REEMPLAZO = revision manual sin CSV.</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RECUPERACIÓN PRIMA PÓLIZA, Recuperaciónprimapóliza, PAGO POR PSE O CODIGO DE BARRAS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>RECU PRIM POLIZA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EXP CARNET</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>1532002509</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EXPEDICION DE CARNET</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EXP CARNET</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CARNET</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>1532002509</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Derecho de de Came Mayor a 180 días</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CARNET</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GC OFICINA</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>1535100020</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>COMMON AREA MAINTENANCE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GC OFICINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ACUED OFICINA</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>1534001605</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Agua y drenaje oficina</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ACUED OFICINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PARQUEADERO OFICINA</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>1532002507</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GTO DE VTA PARQUEADEROS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PARQUEADERO OFICINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RF OFICINA</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>1535100000</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ARRIENDOS INMUEBLES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>RF OFICINA</t>
         </is>
       </c>
     </row>

</xml_diff>